<commit_message>
add text similarity comparison to the edge cases
</commit_message>
<xml_diff>
--- a/data/edge_case/comapre-models.xlsx
+++ b/data/edge_case/comapre-models.xlsx
@@ -308,7 +308,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -402,14 +402,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1720,58 +1712,58 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="24" t="s">
+      <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="24" t="s">
+      <c r="E2" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="25" t="n">
+      <c r="C3" s="13" t="n">
         <v>0.934809067396927</v>
       </c>
-      <c r="D3" s="25" t="n">
+      <c r="D3" s="13" t="n">
         <v>0.912140575079872</v>
       </c>
-      <c r="E3" s="25" t="n">
+      <c r="E3" s="13" t="n">
         <v>0.966453674121406</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="25" t="n">
+      <c r="C4" s="13" t="n">
         <v>0.913501573468894</v>
       </c>
-      <c r="D4" s="25" t="n">
+      <c r="D4" s="13" t="n">
         <v>0.956275720164609</v>
       </c>
-      <c r="E4" s="25" t="n">
+      <c r="E4" s="13" t="n">
         <v>0.880144032921811</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="25" t="n">
+      <c r="C5" s="13" t="n">
         <v>0.427392739273927</v>
       </c>
-      <c r="D5" s="25" t="n">
+      <c r="D5" s="13" t="n">
         <v>0.346534653465347</v>
       </c>
-      <c r="E5" s="25" t="n">
+      <c r="E5" s="13" t="n">
         <v>0.603960396039604</v>
       </c>
     </row>

</xml_diff>